<commit_message>
feat: activate sloth adventure pricing and estimator
Sloth Adventure (slothadventure.html) is now an approved ACTIVE
product, superseding the earlier rule that this page must remain
untouched. It is now included in tour-pricing.json, the Smart Quote
Estimator, its own detail-page pricing, and the /tours catalog, the
same as every other active tour.

Approved commercial pricing (Zone Adjustment Applies = NO):
- Classic: 2 pax $310 / 3 pax $250 / 4+ pax $225 p.p.
- Plus:    2 pax $325 / 3 pax $270 / 4+ pax $240 p.p.

Public starting price: From $225 p.p. for groups of 4+ guests.

tour-pricing.json is now 33 tours (32 ACTIVE + 1 MANUAL QUOTE,
ostionalturtles), pricing_version sha256-b4bfe8a17e5bb3ca.
tour-generator.ps1's scope guard and tours-catalog-pricing-sync.ps1's
completeness guard are both updated to reflect 0 intentionally
excluded tours and 32 ACTIVE catalog cards.

JSON-LD, sitemap, robots and llms are unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
+++ b/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
@@ -635,8 +635,17 @@
       <c r="B10" t="str">
         <v>Classic</v>
       </c>
+      <c r="C10">
+        <v>310</v>
+      </c>
+      <c r="D10">
+        <v>250</v>
+      </c>
+      <c r="E10">
+        <v>225</v>
+      </c>
       <c r="I10" t="str">
-        <v>PENDING REDISTRIBUTION: legacy combined-row rates were $310 (2pax) / $250 (3pax) / $225 (4+pax) p.p. before this tour was split into Classic/Plus. Not assigned to either option -- do not use until confirmed by ops.</v>
+        <v>Confirmed by ops -- Classic $310/$250/$225 p.p., Plus $325/$270/$240 p.p.</v>
       </c>
       <c r="J10" t="str">
         <v>https://wildpapagayo.com/tours/slothadventure.html</v>
@@ -647,8 +656,11 @@
       <c r="L10" t="str">
         <v>classic</v>
       </c>
+      <c r="M10" t="str">
+        <v>NO</v>
+      </c>
       <c r="N10" t="str">
-        <v>INACTIVE</v>
+        <v>ACTIVE</v>
       </c>
     </row>
     <row r="11">
@@ -1849,8 +1861,17 @@
       <c r="B47" t="str">
         <v>Plus</v>
       </c>
+      <c r="C47">
+        <v>325</v>
+      </c>
+      <c r="D47">
+        <v>270</v>
+      </c>
+      <c r="E47">
+        <v>240</v>
+      </c>
       <c r="I47" t="str">
-        <v>PENDING REDISTRIBUTION: legacy combined-row rates were $310 (2pax) / $250 (3pax) / $225 (4+pax) p.p. before this tour was split into Classic/Plus. Not assigned to either option -- do not use until confirmed by ops.</v>
+        <v>Confirmed by ops -- Classic $310/$250/$225 p.p., Plus $325/$270/$240 p.p.</v>
       </c>
       <c r="J47" t="str">
         <v>https://wildpapagayo.com/tours/slothadventure.html</v>
@@ -1861,8 +1882,11 @@
       <c r="L47" t="str">
         <v>plus</v>
       </c>
+      <c r="M47" t="str">
+        <v>NO</v>
+      </c>
       <c r="N47" t="str">
-        <v>INACTIVE</v>
+        <v>ACTIVE</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content(pricing): enable zone adjustments catalog-wide, update Celeste River and Arenal Hanging Bridges
Business-confirmed Excel update: "Zone Adjustment Applies" set to YES
across all 33 tours/43 options in Precios Tours (previously only
per-tour, mostly NO), so the Smart Quote Estimator now applies each
tour's own Zone A/B/C surcharge instead of ignoring it regardless of
the amount entered. Also includes: Celeste River base price lowered
from $300/$240/$215 to $270/$220/$185 (full-experience) plus a new
+$25 Zone C adjustment; Arenal Hanging Bridges gains a new +$30 Zone C
adjustment (both classic and plus); Buena Vista Mega Combo's Zone A
adjustment removed (was $0).

Regenerated via node knowledge/pricing/excel-to-pricing.js, then
tour-generator.ps1, tours-catalog-pricing-sync.ps1 and
recommendation-engine.ps1. content-link-validator.ps1: 0 issues.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
+++ b/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Desktop\Tico 10\wild-papagayo\knowledge\pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CCC6FDD-9F94-4E4F-98CE-948282829263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2AA4D8-9AE1-4DCC-AF12-53D10CB20ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="164">
   <si>
     <t>Matriz maestra de precios — Wild Papagayo</t>
   </si>
@@ -87,9 +87,6 @@
     <t>full-experience</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
     <t>ACTIVE</t>
   </si>
   <si>
@@ -514,6 +511,9 @@
   </si>
   <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>YES</t>
   </si>
 </sst>
 </file>
@@ -1001,18 +1001,18 @@
         <v>20</v>
       </c>
       <c r="M5" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
         <v>23</v>
-      </c>
-      <c r="B6" t="s">
-        <v>24</v>
       </c>
       <c r="C6">
         <v>470</v>
@@ -1027,30 +1027,30 @@
         <v>30</v>
       </c>
       <c r="I6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" t="s">
         <v>25</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>26</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>27</v>
       </c>
-      <c r="L6" t="s">
-        <v>28</v>
-      </c>
       <c r="M6" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7">
         <v>500</v>
@@ -1065,27 +1065,27 @@
         <v>30</v>
       </c>
       <c r="I7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" t="s">
         <v>30</v>
       </c>
-      <c r="J7" t="s">
-        <v>26</v>
-      </c>
-      <c r="K7" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" t="s">
-        <v>31</v>
-      </c>
       <c r="M7" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
@@ -1106,24 +1106,24 @@
         <v>18</v>
       </c>
       <c r="K8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L8" t="s">
         <v>20</v>
       </c>
       <c r="M8" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
         <v>34</v>
-      </c>
-      <c r="B9" t="s">
-        <v>35</v>
       </c>
       <c r="C9">
         <v>355</v>
@@ -1134,34 +1134,31 @@
       <c r="E9">
         <v>275</v>
       </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
       <c r="I9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J9" t="s">
         <v>18</v>
       </c>
       <c r="K9" t="s">
+        <v>36</v>
+      </c>
+      <c r="L9" t="s">
         <v>37</v>
       </c>
-      <c r="L9" t="s">
-        <v>38</v>
-      </c>
       <c r="M9" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>310</v>
@@ -1173,30 +1170,30 @@
         <v>225</v>
       </c>
       <c r="I10" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" t="s">
         <v>40</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>41</v>
       </c>
-      <c r="K10" t="s">
-        <v>42</v>
-      </c>
       <c r="L10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M10" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11">
         <v>565</v>
@@ -1208,30 +1205,30 @@
         <v>410</v>
       </c>
       <c r="I11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" t="s">
         <v>44</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>45</v>
       </c>
-      <c r="K11" t="s">
-        <v>46</v>
-      </c>
       <c r="L11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M11" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12">
         <v>585</v>
@@ -1243,27 +1240,27 @@
         <v>430</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J12" t="s">
+        <v>44</v>
+      </c>
+      <c r="K12" t="s">
         <v>45</v>
       </c>
-      <c r="K12" t="s">
-        <v>46</v>
-      </c>
       <c r="L12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M12" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
         <v>17</v>
@@ -1281,21 +1278,21 @@
         <v>18</v>
       </c>
       <c r="K13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L13" t="s">
         <v>20</v>
       </c>
       <c r="M13" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B14" t="s">
         <v>17</v>
@@ -1313,24 +1310,24 @@
         <v>18</v>
       </c>
       <c r="K14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L14" t="s">
         <v>20</v>
       </c>
       <c r="M14" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>480</v>
@@ -1342,30 +1339,30 @@
         <v>330</v>
       </c>
       <c r="I15" t="s">
+        <v>52</v>
+      </c>
+      <c r="J15" t="s">
         <v>53</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>54</v>
       </c>
-      <c r="K15" t="s">
-        <v>55</v>
-      </c>
       <c r="L15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M15" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16">
         <v>480</v>
@@ -1377,27 +1374,27 @@
         <v>330</v>
       </c>
       <c r="I16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J16" t="s">
+        <v>53</v>
+      </c>
+      <c r="K16" t="s">
         <v>54</v>
       </c>
-      <c r="K16" t="s">
-        <v>55</v>
-      </c>
       <c r="L16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M16" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B17" t="s">
         <v>17</v>
@@ -1415,21 +1412,21 @@
         <v>18</v>
       </c>
       <c r="K17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L17" t="s">
         <v>20</v>
       </c>
       <c r="M17" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
         <v>17</v>
@@ -1447,21 +1444,21 @@
         <v>18</v>
       </c>
       <c r="K18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L18" t="s">
         <v>20</v>
       </c>
       <c r="M18" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
         <v>17</v>
@@ -1479,21 +1476,21 @@
         <v>18</v>
       </c>
       <c r="K19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L19" t="s">
         <v>20</v>
       </c>
       <c r="M19" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
         <v>17</v>
@@ -1511,24 +1508,24 @@
         <v>18</v>
       </c>
       <c r="K20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L20" t="s">
         <v>20</v>
       </c>
       <c r="M20" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21">
         <v>330</v>
@@ -1540,30 +1537,30 @@
         <v>250</v>
       </c>
       <c r="I21" t="s">
+        <v>65</v>
+      </c>
+      <c r="J21" t="s">
         <v>66</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>67</v>
       </c>
-      <c r="K21" t="s">
-        <v>68</v>
-      </c>
       <c r="L21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M21" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C22">
         <v>350</v>
@@ -1575,30 +1572,30 @@
         <v>270</v>
       </c>
       <c r="I22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J22" t="s">
+        <v>66</v>
+      </c>
+      <c r="K22" t="s">
         <v>67</v>
       </c>
-      <c r="K22" t="s">
-        <v>68</v>
-      </c>
       <c r="L22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M22" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23">
         <v>320</v>
@@ -1610,30 +1607,30 @@
         <v>240</v>
       </c>
       <c r="I23" t="s">
+        <v>70</v>
+      </c>
+      <c r="J23" t="s">
         <v>71</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>72</v>
       </c>
-      <c r="K23" t="s">
-        <v>73</v>
-      </c>
       <c r="L23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M23" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24">
         <v>340</v>
@@ -1645,27 +1642,27 @@
         <v>260</v>
       </c>
       <c r="I24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J24" t="s">
+        <v>71</v>
+      </c>
+      <c r="K24" t="s">
         <v>72</v>
       </c>
-      <c r="K24" t="s">
-        <v>73</v>
-      </c>
       <c r="L24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M24" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B25" t="s">
         <v>17</v>
@@ -1686,21 +1683,21 @@
         <v>18</v>
       </c>
       <c r="K25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L25" t="s">
         <v>20</v>
       </c>
       <c r="M25" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
         <v>17</v>
@@ -1709,21 +1706,24 @@
         <v>18</v>
       </c>
       <c r="K26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L26" t="s">
         <v>20</v>
       </c>
+      <c r="M26" t="s">
+        <v>163</v>
+      </c>
       <c r="N26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27">
         <v>330</v>
@@ -1735,30 +1735,30 @@
         <v>250</v>
       </c>
       <c r="I27" t="s">
+        <v>80</v>
+      </c>
+      <c r="J27" t="s">
         <v>81</v>
       </c>
-      <c r="J27" t="s">
+      <c r="K27" t="s">
         <v>82</v>
       </c>
-      <c r="K27" t="s">
-        <v>83</v>
-      </c>
       <c r="L27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M27" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C28">
         <v>350</v>
@@ -1770,27 +1770,27 @@
         <v>270</v>
       </c>
       <c r="I28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J28" t="s">
+        <v>81</v>
+      </c>
+      <c r="K28" t="s">
         <v>82</v>
       </c>
-      <c r="K28" t="s">
-        <v>83</v>
-      </c>
       <c r="L28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M28" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B29" t="s">
         <v>17</v>
@@ -1808,21 +1808,21 @@
         <v>18</v>
       </c>
       <c r="K29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L29" t="s">
         <v>20</v>
       </c>
       <c r="M29" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B30" t="s">
         <v>17</v>
@@ -1840,24 +1840,24 @@
         <v>18</v>
       </c>
       <c r="K30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L30" t="s">
         <v>20</v>
       </c>
       <c r="M30" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C31">
         <v>325</v>
@@ -1869,30 +1869,30 @@
         <v>255</v>
       </c>
       <c r="I31" t="s">
+        <v>89</v>
+      </c>
+      <c r="J31" t="s">
         <v>90</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>91</v>
       </c>
-      <c r="K31" t="s">
-        <v>92</v>
-      </c>
       <c r="L31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M31" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N31" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32">
         <v>325</v>
@@ -1904,27 +1904,27 @@
         <v>255</v>
       </c>
       <c r="I32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J32" t="s">
+        <v>90</v>
+      </c>
+      <c r="K32" t="s">
         <v>91</v>
       </c>
-      <c r="K32" t="s">
-        <v>92</v>
-      </c>
       <c r="L32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M32" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B33" t="s">
         <v>17</v>
@@ -1942,21 +1942,21 @@
         <v>18</v>
       </c>
       <c r="K33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L33" t="s">
         <v>20</v>
       </c>
       <c r="M33" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B34" t="s">
         <v>17</v>
@@ -1974,21 +1974,21 @@
         <v>18</v>
       </c>
       <c r="K34" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L34" t="s">
         <v>20</v>
       </c>
       <c r="M34" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B35" t="s">
         <v>17</v>
@@ -2006,21 +2006,21 @@
         <v>18</v>
       </c>
       <c r="K35" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L35" t="s">
         <v>20</v>
       </c>
       <c r="M35" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B36" t="s">
         <v>17</v>
@@ -2038,24 +2038,24 @@
         <v>18</v>
       </c>
       <c r="K36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L36" t="s">
         <v>20</v>
       </c>
       <c r="M36" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37">
         <v>285</v>
@@ -2067,30 +2067,30 @@
         <v>190</v>
       </c>
       <c r="I37" t="s">
+        <v>102</v>
+      </c>
+      <c r="J37" t="s">
         <v>103</v>
       </c>
-      <c r="J37" t="s">
+      <c r="K37" t="s">
         <v>104</v>
       </c>
-      <c r="K37" t="s">
-        <v>105</v>
-      </c>
       <c r="L37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M37" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C38">
         <v>345</v>
@@ -2102,27 +2102,27 @@
         <v>285</v>
       </c>
       <c r="I38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J38" t="s">
+        <v>103</v>
+      </c>
+      <c r="K38" t="s">
         <v>104</v>
       </c>
-      <c r="K38" t="s">
-        <v>105</v>
-      </c>
       <c r="L38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M38" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N38" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B39" t="s">
         <v>17</v>
@@ -2140,21 +2140,21 @@
         <v>18</v>
       </c>
       <c r="K39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L39" t="s">
         <v>20</v>
       </c>
       <c r="M39" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B40" t="s">
         <v>17</v>
@@ -2172,21 +2172,21 @@
         <v>18</v>
       </c>
       <c r="K40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L40" t="s">
         <v>20</v>
       </c>
       <c r="M40" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B41" t="s">
         <v>17</v>
@@ -2204,21 +2204,21 @@
         <v>18</v>
       </c>
       <c r="K41" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L41" t="s">
         <v>20</v>
       </c>
       <c r="M41" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B42" t="s">
         <v>17</v>
@@ -2236,24 +2236,24 @@
         <v>18</v>
       </c>
       <c r="K42" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L42" t="s">
         <v>20</v>
       </c>
       <c r="M42" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N42" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43">
         <v>275</v>
@@ -2265,30 +2265,30 @@
         <v>220</v>
       </c>
       <c r="I43" t="s">
+        <v>115</v>
+      </c>
+      <c r="J43" t="s">
         <v>116</v>
       </c>
-      <c r="J43" t="s">
+      <c r="K43" t="s">
         <v>117</v>
       </c>
-      <c r="K43" t="s">
-        <v>118</v>
-      </c>
       <c r="L43" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M43" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N43" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C44">
         <v>395</v>
@@ -2300,27 +2300,27 @@
         <v>340</v>
       </c>
       <c r="I44" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J44" t="s">
+        <v>116</v>
+      </c>
+      <c r="K44" t="s">
         <v>117</v>
       </c>
-      <c r="K44" t="s">
-        <v>118</v>
-      </c>
       <c r="L44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M44" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B45" t="s">
         <v>17</v>
@@ -2338,21 +2338,21 @@
         <v>18</v>
       </c>
       <c r="K45" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L45" t="s">
         <v>20</v>
       </c>
       <c r="M45" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N45" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B46" t="s">
         <v>17</v>
@@ -2367,30 +2367,30 @@
         <v>325</v>
       </c>
       <c r="I46" t="s">
+        <v>122</v>
+      </c>
+      <c r="J46" t="s">
         <v>123</v>
       </c>
-      <c r="J46" t="s">
+      <c r="K46" t="s">
         <v>124</v>
-      </c>
-      <c r="K46" t="s">
-        <v>125</v>
       </c>
       <c r="L46" t="s">
         <v>20</v>
       </c>
       <c r="M46" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N46" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C47">
         <v>325</v>
@@ -2402,22 +2402,22 @@
         <v>240</v>
       </c>
       <c r="I47" t="s">
+        <v>39</v>
+      </c>
+      <c r="J47" t="s">
         <v>40</v>
       </c>
-      <c r="J47" t="s">
+      <c r="K47" t="s">
         <v>41</v>
       </c>
-      <c r="K47" t="s">
-        <v>42</v>
-      </c>
       <c r="L47" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="M47" t="s">
-        <v>21</v>
+        <v>163</v>
       </c>
       <c r="N47" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2427,7 +2427,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:N4 A9:N24 A5:B5 F5:G5 N5 I5:L5 A26:N47 A25:B25 F25:G25 I25:N25 A6:G6 I6:N6 A7:G7 I7:N7 A8:B8 F8:G8 I8:N8" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:N4 A10:L24 A5:B5 F5:G5 N5 I5:L5 A26:L47 A25:B25 F25:G25 I25:L25 A6:G6 I6:L6 A7:G7 I7:L7 A8:B8 F8:G8 I8:L8 N9:N24 N26:N47 N25 N6 N7 N8 A9:E9 G9:L9" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2444,7 +2444,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2452,7 +2452,7 @@
     </row>
     <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2460,13 +2460,13 @@
     </row>
     <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
         <v>128</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>129</v>
-      </c>
-      <c r="C4" t="s">
-        <v>130</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -2474,104 +2474,104 @@
     </row>
     <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B5" t="s">
         <v>131</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>132</v>
-      </c>
-      <c r="C5" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" t="s">
         <v>134</v>
       </c>
-      <c r="B6" t="s">
-        <v>135</v>
-      </c>
       <c r="C6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C8" t="s">
         <v>132</v>
-      </c>
-      <c r="C8" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" t="s">
         <v>132</v>
-      </c>
-      <c r="C9" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" t="s">
         <v>132</v>
-      </c>
-      <c r="C10" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
+        <v>131</v>
+      </c>
+      <c r="C11" t="s">
         <v>132</v>
-      </c>
-      <c r="C11" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" t="s">
-        <v>163</v>
-      </c>
       <c r="C12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>140</v>
+      </c>
+      <c r="B13" t="s">
         <v>141</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>142</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>143</v>
-      </c>
-      <c r="D13" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -2593,72 +2593,72 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" t="s">
         <v>146</v>
-      </c>
-      <c r="B3" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B4" t="s">
         <v>148</v>
-      </c>
-      <c r="B4" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" t="s">
         <v>150</v>
-      </c>
-      <c r="B5" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B6" t="s">
         <v>152</v>
-      </c>
-      <c r="B6" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>153</v>
+      </c>
+      <c r="B7" t="s">
         <v>154</v>
-      </c>
-      <c r="B7" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" t="s">
         <v>156</v>
-      </c>
-      <c r="B8" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" t="s">
         <v>158</v>
-      </c>
-      <c r="B9" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B10" t="s">
         <v>160</v>
-      </c>
-      <c r="B10" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
content(pricing): update confirmed Zone C tour adjustments
Owner-confirmed Zone C surcharge increase on 5 options: Costa Rica
Highlights full-experience, Arenal Hanging Bridges classic/plus,
Celeste River full-experience, and Oropendola Hot Springs
full-experience ($25->$50 or $30->$60). Base per-person prices
(pp_2/pp_3/pp_4plus) and Zone A/B adjustments are unchanged.
Celeste River has zone_adjustment_applies=NO, so its Zone C value is
not consulted by the estimator and this change has no customer-facing
effect for that tour.

Regenerated via npm run pricing:convert from the Excel source. 0
other cells changed in the Excel; 0 base-price drift; 0 Offer.price
changes in generated schema; 0 commercial changes in
recommendations.json (timestamp-only regen reverted, not committed).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
+++ b/knowledge/pricing/Matriz_Cotizador_Wild_Papagayo_Catalogo_Completo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Desktop\Tico 10\wild-papagayo\knowledge\pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74992F94-1446-4F3C-9D8A-BC5113482C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51B882A1-AA36-4793-B461-934EA8EC2413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -998,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="J5" t="s">
         <v>18</v>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="I6" t="s">
         <v>25</v>
@@ -1083,7 +1083,7 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="I7" t="s">
         <v>30</v>
@@ -1127,7 +1127,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="J8" t="s">
         <v>18</v>
@@ -1854,7 +1854,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="J25" t="s">
         <v>18</v>

</xml_diff>